<commit_message>
final testing point after adding api
</commit_message>
<xml_diff>
--- a/output/test_bom_cleaned_bom.xlsx
+++ b/output/test_bom_cleaned_bom.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Warnings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clean_BOM'!$A$1:$R$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clean_BOM'!$A$1:$X$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review_Items'!$A$1:$X$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Column_Mapping'!$A$1:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,16 +24,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -452,104 +441,140 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>designators</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>qty_per_board</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>build_quantity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>overage_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>required_qty</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mpn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>supplier_part_number</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>subtotal</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>lifecycle_status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>build_multiplier</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>selected_supplier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>supplier_order_qty</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>mouser_stock</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>digikey_stock</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>sourcing_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sourcing_notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -566,13 +591,13 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G2" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -592,13 +617,43 @@
       <c r="Q2" t="inlineStr">
         <is>
           <t>clean</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Mouser</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>sourced_mouser</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Mouser can cover full required quantity.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -615,13 +670,13 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G3" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -641,13 +696,33 @@
       <c r="Q3" t="inlineStr">
         <is>
           <t>clean</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -664,13 +739,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -690,13 +765,33 @@
       <c r="Q4" t="inlineStr">
         <is>
           <t>clean</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -713,13 +808,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G5" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -741,9 +836,29 @@
           <t>clean</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R5"/>
+  <autoFilter ref="A1:X5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -754,19 +869,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
@@ -775,101 +890,345 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>designators</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>qty_per_board</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>build_quantity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>overage_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>required_qty</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mpn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>supplier_part_number</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>subtotal</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>lifecycle_status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>build_multiplier</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>selected_supplier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>supplier_order_qty</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>mouser_stock</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>digikey_stock</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>sourcing_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sourcing_notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>test_BOM.CSV</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>C1 C2</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Murata</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>GRM188R71C105KA12D</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1uF Capacitor 16V 0603</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>test_BOM.CSV</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>STMicroelectronics</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>STM32F411CEU6</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Microcontroller</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>test_BOM.CSV</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TDK</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>VLS6045EX-100M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Inductor 10uH</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:X4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -891,27 +1250,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>standard_field</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>selected_column</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>candidate_columns</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -920,7 +1279,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -947,7 +1306,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -974,7 +1333,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1001,7 +1360,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1028,7 +1387,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1055,7 +1414,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1072,7 +1431,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1089,7 +1448,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1106,7 +1465,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1123,7 +1482,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>test_bom.csv</t>
+          <t>test_BOM.CSV</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1160,27 +1519,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>message</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>value</t>
         </is>

</xml_diff>

<commit_message>
check point mouser connects
</commit_message>
<xml_diff>
--- a/output/test_bom_cleaned_bom.xlsx
+++ b/output/test_bom_cleaned_bom.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Warnings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clean_BOM'!$A$1:$R$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clean_BOM'!$A$1:$X$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review_Items'!$A$1:$X$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Column_Mapping'!$A$1:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,16 +24,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -452,97 +441,133 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>designators</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>qty_per_board</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>build_quantity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>overage_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>required_qty</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mpn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>supplier_part_number</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>subtotal</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>lifecycle_status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>build_multiplier</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>selected_supplier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>supplier_order_qty</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>mouser_stock</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>digikey_stock</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>sourcing_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sourcing_notes</t>
         </is>
       </c>
     </row>
@@ -569,7 +594,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G2" t="n">
         <v>4</v>
@@ -594,6 +619,36 @@
           <t>clean</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Mouser</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>3702426</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>sourced_mouser</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Mouser can cover full required quantity.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -618,7 +673,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
@@ -643,6 +698,26 @@
           <t>clean</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -667,7 +742,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
@@ -692,6 +767,36 @@
           <t>clean</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Mouser</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>sourced_mouser</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Mouser can cover full required quantity.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -716,7 +821,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
@@ -741,9 +846,39 @@
           <t>clean</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Mouser</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>4590</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>sourced_mouser</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Mouser can cover full required quantity.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R5"/>
+  <autoFilter ref="A1:X5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -754,10 +889,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -765,8 +900,8 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
@@ -775,101 +910,207 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>designators</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>qty_per_board</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>build_quantity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>overage_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>required_qty</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mpn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>supplier_part_number</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>subtotal</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>lifecycle_status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>build_multiplier</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>selected_supplier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>supplier_order_qty</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>mouser_stock</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>digikey_stock</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>sourcing_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sourcing_notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>test_bom.csv</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>C1 C2</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Murata</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>GRM188R71C105KA12D</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1uF Capacitor 16V 0603</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>check_wall_inventory</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Neither Mouser nor DigiKey can cover full required quantity.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:X2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -891,27 +1132,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>standard_field</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>selected_column</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>candidate_columns</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1160,27 +1401,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>message</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>value</t>
         </is>

</xml_diff>

<commit_message>
need some more work trying to add mouser
</commit_message>
<xml_diff>
--- a/output/test_bom_cleaned_bom.xlsx
+++ b/output/test_bom_cleaned_bom.xlsx
@@ -24,16 +24,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -44,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -52,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,122 +450,122 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>designators</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>qty_per_board</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>build_quantity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>overage_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>required_qty</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mpn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>supplier_part_number</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>subtotal</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>lifecycle_status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>build_multiplier</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>selected_supplier</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>supplier_order_qty</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>mouser_stock</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>digikey_stock</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>sourcing_status</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>sourcing_notes</t>
         </is>
@@ -626,6 +614,11 @@
           <t>10k Resistor 1% 0603</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0.004</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>clean</t>
@@ -638,7 +631,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -648,7 +641,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>10838928</t>
+          <t>10234542</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -774,6 +767,11 @@
           <t>Microcontroller</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>6.63</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr">
         <is>
           <t>clean</t>
@@ -786,7 +784,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -796,7 +794,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>3936</t>
+          <t>3401</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -853,6 +851,11 @@
           <t>Inductor 10uH</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0.18404</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
           <t>clean</t>
@@ -865,7 +868,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -875,7 +878,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>44737</t>
+          <t>44532</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -931,122 +934,122 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>designators</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>qty_per_board</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>build_quantity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>overage_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>required_qty</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mpn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>supplier_part_number</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>subtotal</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>lifecycle_status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>build_multiplier</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>selected_supplier</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>supplier_order_qty</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>mouser_stock</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>digikey_stock</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>sourcing_status</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>sourcing_notes</t>
         </is>
@@ -1144,27 +1147,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>standard_field</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>selected_column</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>candidate_columns</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1413,27 +1416,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>source_row</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>message</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>value</t>
         </is>

</xml_diff>